<commit_message>
Fix: Round 4 QA beta feedback issues (Say&Check, WordFamily, SRS, and assets)
</commit_message>
<xml_diff>
--- a/아바타 체크용 엑셀시트.xlsx
+++ b/아바타 체크용 엑셀시트.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\origi\Antigravity-workspaces\Main_English\phonics-app\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="8_{DFA04FE8-4F07-42E1-AE6E-E1EF8EE2BD71}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{E94FFE1A-C0D8-4ED2-9AAF-6D6E2A90FB14}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-98" yWindow="-98" windowWidth="21795" windowHeight="12975" xr2:uid="{51658058-8315-A640-B733-1DFC39D6EEC8}"/>
   </bookViews>
@@ -36,7 +36,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="206" uniqueCount="116">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="210" uniqueCount="118">
   <si>
     <t>No.</t>
   </si>
@@ -384,6 +384,13 @@
   </si>
   <si>
     <t>이상있음</t>
+  </si>
+  <si>
+    <t>기타</t>
+  </si>
+  <si>
+    <t>뒷발음이 일부 파일에 담김</t>
+    <phoneticPr fontId="4" type="noConversion"/>
   </si>
 </sst>
 </file>
@@ -1424,10 +1431,18 @@
       <c r="C38" s="9" t="s">
         <v>48</v>
       </c>
-      <c r="D38" s="8"/>
-      <c r="E38" s="8"/>
-      <c r="F38" s="8"/>
-      <c r="G38" s="10"/>
+      <c r="D38" s="8" t="s">
+        <v>114</v>
+      </c>
+      <c r="E38" s="8" t="s">
+        <v>115</v>
+      </c>
+      <c r="F38" s="8" t="s">
+        <v>116</v>
+      </c>
+      <c r="G38" s="10" t="s">
+        <v>117</v>
+      </c>
     </row>
     <row r="39" spans="1:7" ht="25.05" customHeight="1" x14ac:dyDescent="0.7">
       <c r="A39" s="8">
@@ -2303,6 +2318,24 @@
 </file>
 
 <file path=customXml/item1.xml><?xml version="1.0" encoding="utf-8"?>
+<?mso-contentType ?>
+<FormTemplates xmlns="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms">
+  <Display>DocumentLibraryForm</Display>
+  <Edit>DocumentLibraryForm</Edit>
+  <New>DocumentLibraryForm</New>
+</FormTemplates>
+</file>
+
+<file path=customXml/item2.xml><?xml version="1.0" encoding="utf-8"?>
+<p:properties xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:xsi="http://www.w3.org/2001/XMLSchema-instance" xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls">
+  <documentManagement>
+    <Document_x0020_Purpose xmlns="f577acbf-5b0b-4b4f-9948-268e97f8d3a4">Informational</Document_x0020_Purpose>
+    <Initiatives xmlns="f577acbf-5b0b-4b4f-9948-268e97f8d3a4"/>
+  </documentManagement>
+</p:properties>
+</file>
+
+<file path=customXml/item3.xml><?xml version="1.0" encoding="utf-8"?>
 <ct:contentTypeSchema xmlns:ct="http://schemas.microsoft.com/office/2006/metadata/contentType" xmlns:ma="http://schemas.microsoft.com/office/2006/metadata/properties/metaAttributes" ct:_="" ma:_="" ma:contentTypeName="Document" ma:contentTypeID="0x010100CD401524DC532D42A0E0ED886331A72B" ma:contentTypeVersion="13" ma:contentTypeDescription="Create a new document." ma:contentTypeScope="" ma:versionID="d936d863d335d354da51eb78ca1ae338">
   <xsd:schema xmlns:xsd="http://www.w3.org/2001/XMLSchema" xmlns:xs="http://www.w3.org/2001/XMLSchema" xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:ns2="f577acbf-5b0b-4b4f-9948-268e97f8d3a4" xmlns:ns3="b1e4d6ee-9f6f-43f8-a618-24f3d84da28f" targetNamespace="http://schemas.microsoft.com/office/2006/metadata/properties" ma:root="true" ma:fieldsID="5fbac08d56b1b04aa33acbc31e882ce9" ns2:_="" ns3:_="">
     <xsd:import namespace="f577acbf-5b0b-4b4f-9948-268e97f8d3a4"/>
@@ -2546,39 +2579,10 @@
 </ct:contentTypeSchema>
 </file>
 
-<file path=customXml/item2.xml><?xml version="1.0" encoding="utf-8"?>
-<p:properties xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:xsi="http://www.w3.org/2001/XMLSchema-instance" xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls">
-  <documentManagement>
-    <Document_x0020_Purpose xmlns="f577acbf-5b0b-4b4f-9948-268e97f8d3a4">Informational</Document_x0020_Purpose>
-    <Initiatives xmlns="f577acbf-5b0b-4b4f-9948-268e97f8d3a4"/>
-  </documentManagement>
-</p:properties>
-</file>
-
-<file path=customXml/item3.xml><?xml version="1.0" encoding="utf-8"?>
-<?mso-contentType ?>
-<FormTemplates xmlns="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms">
-  <Display>DocumentLibraryForm</Display>
-  <Edit>DocumentLibraryForm</Edit>
-  <New>DocumentLibraryForm</New>
-</FormTemplates>
-</file>
-
 <file path=customXml/itemProps1.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{2426A393-DB36-49FF-B8B1-6D5559B7ABFC}">
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{1F48E296-90D9-4A92-A29D-759F46DCA7D9}">
   <ds:schemaRefs>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/contentType"/>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/properties/metaAttributes"/>
-    <ds:schemaRef ds:uri="http://www.w3.org/2001/XMLSchema"/>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/properties"/>
-    <ds:schemaRef ds:uri="f577acbf-5b0b-4b4f-9948-268e97f8d3a4"/>
-    <ds:schemaRef ds:uri="b1e4d6ee-9f6f-43f8-a618-24f3d84da28f"/>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/documentManagement/types"/>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
-    <ds:schemaRef ds:uri="http://schemas.openxmlformats.org/package/2006/metadata/core-properties"/>
-    <ds:schemaRef ds:uri="http://purl.org/dc/elements/1.1/"/>
-    <ds:schemaRef ds:uri="http://purl.org/dc/terms/"/>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/internal/obd"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms"/>
   </ds:schemaRefs>
 </ds:datastoreItem>
 </file>
@@ -2601,9 +2605,20 @@
 </file>
 
 <file path=customXml/itemProps3.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{1F48E296-90D9-4A92-A29D-759F46DCA7D9}">
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{2426A393-DB36-49FF-B8B1-6D5559B7ABFC}">
   <ds:schemaRefs>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/contentType"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/properties/metaAttributes"/>
+    <ds:schemaRef ds:uri="http://www.w3.org/2001/XMLSchema"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/properties"/>
+    <ds:schemaRef ds:uri="f577acbf-5b0b-4b4f-9948-268e97f8d3a4"/>
+    <ds:schemaRef ds:uri="b1e4d6ee-9f6f-43f8-a618-24f3d84da28f"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/documentManagement/types"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
+    <ds:schemaRef ds:uri="http://schemas.openxmlformats.org/package/2006/metadata/core-properties"/>
+    <ds:schemaRef ds:uri="http://purl.org/dc/elements/1.1/"/>
+    <ds:schemaRef ds:uri="http://purl.org/dc/terms/"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/internal/obd"/>
   </ds:schemaRefs>
 </ds:datastoreItem>
 </file>
</xml_diff>